<commit_message>
continuing where i left off fixed processor and modified appropriate function to move diagonally witha trapozoidal i.e. ramp movement.
</commit_message>
<xml_diff>
--- a/Gcode_Commands.xlsx
+++ b/Gcode_Commands.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\varga\Documents\PlatformIO\Projects\GantryCode\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{96B224CA-C261-4F14-AE49-78E3EB108A38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B9B764C-F10F-41E4-B4A7-42B20427DE8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="24196" windowHeight="14476" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,12 +16,11 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="124519"/>
-  <fileRecoveryPr repairLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="81">
   <si>
     <t>Command</t>
   </si>
@@ -252,6 +251,18 @@
   </si>
   <si>
     <t>M18 X Y</t>
+  </si>
+  <si>
+    <t>G20</t>
+  </si>
+  <si>
+    <t>change units to inches</t>
+  </si>
+  <si>
+    <t>G21</t>
+  </si>
+  <si>
+    <t>change units to mm</t>
   </si>
 </sst>
 </file>
@@ -744,7 +755,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr defaultRowHeight="24" customHeight="1" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="11.3984375" bestFit="1" customWidth="1"/>
@@ -838,240 +849,260 @@
       </c>
     </row>
     <row r="7" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A7" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="B7" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="C7" s="10" t="s">
-        <v>51</v>
-      </c>
-      <c r="D7" s="11" t="s">
-        <v>67</v>
-      </c>
+      <c r="A7" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="C7" s="6"/>
+      <c r="D7" s="7"/>
     </row>
     <row r="8" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A8" s="9" t="s">
-        <v>10</v>
-      </c>
-      <c r="B8" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="C8" s="10" t="s">
-        <v>52</v>
-      </c>
-      <c r="D8" s="11" t="s">
-        <v>10</v>
-      </c>
+      <c r="A8" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="B8" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="C8" s="6"/>
+      <c r="D8" s="7"/>
     </row>
     <row r="9" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A9" s="9" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B9" s="8" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>11</v>
+        <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A10" s="9" t="s">
+        <v>10</v>
+      </c>
+      <c r="B10" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="D10" s="11" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A11" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B11" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C11" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="D11" s="11" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A12" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B12" s="8" t="s">
         <v>34</v>
       </c>
-      <c r="C10" s="10" t="s">
+      <c r="C12" s="10" t="s">
         <v>53</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="D12" s="11" t="s">
         <v>68</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A11" s="12" t="s">
-        <v>13</v>
-      </c>
-      <c r="B11" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="C11" s="14" t="s">
-        <v>54</v>
-      </c>
-      <c r="D11" s="15" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A12" s="12" t="s">
-        <v>14</v>
-      </c>
-      <c r="B12" s="13" t="s">
-        <v>36</v>
-      </c>
-      <c r="C12" s="14" t="s">
-        <v>55</v>
-      </c>
-      <c r="D12" s="15" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A13" s="12" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A14" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="D14" s="7" t="s">
-        <v>72</v>
+      <c r="A14" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="C14" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="D14" s="15" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A15" s="12" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
     </row>
     <row r="16" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A16" s="4" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A17" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="D17" s="7" t="s">
-        <v>19</v>
+      <c r="A17" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="C17" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="D17" s="15" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A18" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A19" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>41</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A20" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B20" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="C18" s="6" t="s">
+      <c r="C20" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="D18" s="7" t="s">
+      <c r="D20" s="7" t="s">
         <v>20</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A19" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="B19" s="13" t="s">
-        <v>43</v>
-      </c>
-      <c r="C19" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="D19" s="15" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="20" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
-      <c r="A20" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="B20" s="13" t="s">
-        <v>44</v>
-      </c>
-      <c r="C20" s="14" t="s">
-        <v>52</v>
-      </c>
-      <c r="D20" s="15" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="21" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A21" s="12" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B21" s="13" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="C21" s="14" t="s">
         <v>52</v>
       </c>
       <c r="D21" s="15" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="22" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A22" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="C22" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="D22" s="15" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A23" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="C23" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="D23" s="15" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.55000000000000004">
+      <c r="A24" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="B22" s="13" t="s">
+      <c r="B24" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="C22" s="14" t="s">
+      <c r="C24" s="14" t="s">
         <v>60</v>
       </c>
-      <c r="D22" s="15" t="s">
+      <c r="D24" s="15" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="23" spans="1:4" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
-      <c r="A23" s="16" t="s">
+    <row r="25" spans="1:4" ht="24" customHeight="1" thickBot="1" x14ac:dyDescent="0.6">
+      <c r="A25" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="B23" s="17" t="s">
+      <c r="B25" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="C23" s="18" t="s">
+      <c r="C25" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="D23" s="19" t="s">
+      <c r="D25" s="19" t="s">
         <v>76</v>
       </c>
     </row>

</xml_diff>